<commit_message>
Update ALiS baseline framework
</commit_message>
<xml_diff>
--- a/tests/ALiS_Baseline/baselines/Modify/DPBH/CCP.xlsx
+++ b/tests/ALiS_Baseline/baselines/Modify/DPBH/CCP.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" firstSheet="4" activeTab="2"/>
+    <workbookView windowWidth="23040" windowHeight="9000" firstSheet="4" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="TC01_Tabs" sheetId="1" r:id="rId1"/>
@@ -486,7 +486,7 @@
     <t>Text</t>
   </si>
   <si>
-    <t>Nevada Business ID is issued by Secretary of State (SoS) through common business registration process using SilverFlume. To find more details about common business registration process Click Here .This always begins with NV followed by 11 numbers.</t>
+    <t>Nevada Business ID is issued by Secretary of State (SoS) through common business registration process using SilverFlume. To find more details about common business registration process Click Here. This always begins with NV followed by 11 numbers.</t>
   </si>
   <si>
     <t>Please click 'Add' to add a new row.</t>
@@ -5441,7 +5441,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="Nevada Business ID is issued by Secretary of State (SoS) through common business registration process using SilverFlume. To find more details about common business registration process Click Here .This always begins with NV followed by 11 numbers."/>
+    <hyperlink ref="C2" r:id="rId1" display="Nevada Business ID is issued by Secretary of State (SoS) through common business registration process using SilverFlume. To find more details about common business registration process Click Here. This always begins with NV followed by 11 numbers."/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>